<commit_message>
feat: add ai工具箱 listing
</commit_message>
<xml_diff>
--- a/ai-api-sites-table.xlsx
+++ b/ai-api-sites-table.xlsx
@@ -1287,7 +1287,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F30"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.81818181818182" defaultRowHeight="14"/>
   <cols>
     <col width="7" customWidth="1" style="9" min="1" max="1"/>
@@ -2057,6 +2057,36 @@
       <c r="F30" s="0" t="inlineStr">
         <is>
           <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>35</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>ai工具箱</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>https://api.aiaiai001.com/sign-up?aff=ahhq</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>GPT</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>实测：邮箱注册 倍率：GPT-Plus-特价 0.1x 邀请：邀请注册双方各得5刀余额 须知：可用5.6sol</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add VC listing
</commit_message>
<xml_diff>
--- a/ai-api-sites-table.xlsx
+++ b/ai-api-sites-table.xlsx
@@ -1287,7 +1287,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F31"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.81818181818182" defaultRowHeight="14"/>
   <cols>
     <col width="7" customWidth="1" style="9" min="1" max="1"/>
@@ -2061,30 +2061,56 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="n">
+      <c r="A31" s="0" t="n">
         <v>35</v>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B31" s="0" t="inlineStr">
         <is>
           <t>ai工具箱</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C31" s="0" t="inlineStr">
         <is>
           <t>https://api.aiaiai001.com/sign-up?aff=ahhq</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D31" s="0" t="inlineStr">
         <is>
           <t>GPT</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
+      <c r="E31" s="0" t="inlineStr">
         <is>
           <t>实测：邮箱注册 倍率：GPT-Plus-特价 0.1x 邀请：邀请注册双方各得5刀余额 须知：可用5.6sol</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr">
+      <c r="F31" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>36</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>VC</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>https://sub.vcnovb.cn/register?aff=SM594AJGQRNR</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>倍率0.01，每天可抽奖，最高5刀</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
         <is>
           <t>2026-07-16</t>
         </is>

</xml_diff>

<commit_message>
feat: add JBB 金贝贝 listing
</commit_message>
<xml_diff>
--- a/ai-api-sites-table.xlsx
+++ b/ai-api-sites-table.xlsx
@@ -1287,7 +1287,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F32"/>
+  <dimension ref="A1:F33"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.81818181818182" defaultRowHeight="14"/>
   <cols>
     <col width="7" customWidth="1" style="9" min="1" max="1"/>
@@ -2091,28 +2091,58 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="n">
+      <c r="A32" s="0" t="n">
         <v>36</v>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B32" s="0" t="inlineStr">
         <is>
           <t>VC</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C32" s="0" t="inlineStr">
         <is>
           <t>https://sub.vcnovb.cn/register?aff=SM594AJGQRNR</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr"/>
-      <c r="E32" t="inlineStr">
+      <c r="D32" s="0" t="inlineStr"/>
+      <c r="E32" s="0" t="inlineStr">
         <is>
           <t>倍率0.01，每天可抽奖，最高5刀</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr">
+      <c r="F32" s="0" t="inlineStr">
         <is>
           <t>2026-07-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>37</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>JBB 金贝贝</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>https://downstream.jbbtoken.cn/sign-up?aff=FfEj</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>GPT</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>进群给2刀；倍率：kiro 0.2x，gpt 0.1x，ccmax 0.5x</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add 启悟流 listing
</commit_message>
<xml_diff>
--- a/ai-api-sites-table.xlsx
+++ b/ai-api-sites-table.xlsx
@@ -1287,7 +1287,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F33"/>
+  <dimension ref="A1:F34"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.81818181818182" defaultRowHeight="14"/>
   <cols>
     <col width="7" customWidth="1" style="9" min="1" max="1"/>
@@ -2117,30 +2117,56 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="n">
+      <c r="A33" s="0" t="n">
         <v>37</v>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B33" s="0" t="inlineStr">
         <is>
           <t>JBB 金贝贝</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C33" s="0" t="inlineStr">
         <is>
           <t>https://downstream.jbbtoken.cn/sign-up?aff=FfEj</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
+      <c r="D33" s="0" t="inlineStr">
         <is>
           <t>GPT</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
+      <c r="E33" s="0" t="inlineStr">
         <is>
           <t>进群给2刀；倍率：kiro 0.2x，gpt 0.1x，ccmax 0.5x</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr">
+      <c r="F33" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>38</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>启悟流</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>https://756777.xyz/register?aff=3R885475B5SZ</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>注册加群领50刀体验卡，充值比例1：10，最低0.049倍率；邀请好友注册并充值满10元，双方各领66刀体验卡；充值100元可获888刀体验卡。</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
         <is>
           <t>2026-07-28</t>
         </is>

</xml_diff>

<commit_message>
feat: add 中专大王 listing
</commit_message>
<xml_diff>
--- a/ai-api-sites-table.xlsx
+++ b/ai-api-sites-table.xlsx
@@ -1287,7 +1287,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F34"/>
+  <dimension ref="A1:F35"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.81818181818182" defaultRowHeight="14"/>
   <cols>
     <col width="7" customWidth="1" style="9" min="1" max="1"/>
@@ -2147,26 +2147,56 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="n">
+      <c r="A34" s="0" t="n">
         <v>38</v>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B34" s="0" t="inlineStr">
         <is>
           <t>启悟流</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C34" s="0" t="inlineStr">
         <is>
           <t>https://756777.xyz/register?aff=3R885475B5SZ</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr"/>
-      <c r="E34" t="inlineStr">
+      <c r="D34" s="0" t="inlineStr"/>
+      <c r="E34" s="0" t="inlineStr">
         <is>
           <t>注册加群领50刀体验卡，充值比例1：10，最低0.049倍率；邀请好友注册并充值满10元，双方各领66刀体验卡；充值100元可获888刀体验卡。</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr">
+      <c r="F34" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>39</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>中专大王</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>http://www.xn--ohq4b780ces0a.xyz/sign-up?aff=aqhj</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>签到;GPT</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>进群领1刀，每天可签到，GPT 0.02x。</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
         <is>
           <t>2026-07-28</t>
         </is>

</xml_diff>

<commit_message>
feat: add CHH listing
</commit_message>
<xml_diff>
--- a/ai-api-sites-table.xlsx
+++ b/ai-api-sites-table.xlsx
@@ -1287,7 +1287,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F35"/>
+  <dimension ref="A1:F36"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.81818181818182" defaultRowHeight="14"/>
   <cols>
     <col width="7" customWidth="1" style="9" min="1" max="1"/>
@@ -2173,30 +2173,56 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="n">
+      <c r="A35" s="0" t="n">
         <v>39</v>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B35" s="0" t="inlineStr">
         <is>
           <t>中专大王</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="C35" s="0" t="inlineStr">
         <is>
           <t>http://www.xn--ohq4b780ces0a.xyz/sign-up?aff=aqhj</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
+      <c r="D35" s="0" t="inlineStr">
         <is>
           <t>签到;GPT</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr">
+      <c r="E35" s="0" t="inlineStr">
         <is>
           <t>进群领1刀，每天可签到，GPT 0.02x。</t>
         </is>
       </c>
-      <c r="F35" t="inlineStr">
+      <c r="F35" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>40</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>CHH</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>https://api.chhlink.xyz/register?aff=4UFN5ZCRNDKV</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr"/>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>进群领50刀。</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
         <is>
           <t>2026-07-28</t>
         </is>

</xml_diff>

<commit_message>
feat: add gorouter listing
</commit_message>
<xml_diff>
--- a/ai-api-sites-table.xlsx
+++ b/ai-api-sites-table.xlsx
@@ -1287,7 +1287,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F36"/>
+  <dimension ref="A1:F37"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.81818181818182" defaultRowHeight="14"/>
   <cols>
     <col width="7" customWidth="1" style="9" min="1" max="1"/>
@@ -2203,28 +2203,58 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="n">
+      <c r="A36" s="0" t="n">
         <v>40</v>
       </c>
-      <c r="B36" t="inlineStr">
+      <c r="B36" s="0" t="inlineStr">
         <is>
           <t>CHH</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C36" s="0" t="inlineStr">
         <is>
           <t>https://api.chhlink.xyz/register?aff=4UFN5ZCRNDKV</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr"/>
-      <c r="E36" t="inlineStr">
+      <c r="D36" s="0" t="inlineStr"/>
+      <c r="E36" s="0" t="inlineStr">
         <is>
           <t>进群领50刀。</t>
         </is>
       </c>
-      <c r="F36" t="inlineStr">
+      <c r="F36" s="0" t="inlineStr">
         <is>
           <t>2026-07-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>41</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>gorouter</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>https://gorouter.app/sign-up?aff=GvWs</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>注册赠送;Claude</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>需要使用 GitHub 注册，注册赠送70刀，可使用 Claude。</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add modelport listing
</commit_message>
<xml_diff>
--- a/ai-api-sites-table.xlsx
+++ b/ai-api-sites-table.xlsx
@@ -1287,7 +1287,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F37"/>
+  <dimension ref="A1:F38"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.81818181818182" defaultRowHeight="14"/>
   <cols>
     <col width="7" customWidth="1" style="9" min="1" max="1"/>
@@ -2229,32 +2229,62 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" t="n">
+      <c r="A37" s="0" t="n">
         <v>41</v>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="B37" s="0" t="inlineStr">
         <is>
           <t>gorouter</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C37" s="0" t="inlineStr">
         <is>
           <t>https://gorouter.app/sign-up?aff=GvWs</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
+      <c r="D37" s="0" t="inlineStr">
         <is>
           <t>注册赠送;Claude</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr">
+      <c r="E37" s="0" t="inlineStr">
         <is>
           <t>需要使用 GitHub 注册，注册赠送70刀，可使用 Claude。</t>
         </is>
       </c>
-      <c r="F37" t="inlineStr">
+      <c r="F37" s="0" t="inlineStr">
         <is>
           <t>2026-07-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>42</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>modelport</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>https://modelport.link/register?aff=KXEDZYFPJTH6</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>GPT</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>进群联系管理员可领取官倍 ¥3 站内体验额度，GPT 0.1x。</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add JuCodex listing
</commit_message>
<xml_diff>
--- a/ai-api-sites-table.xlsx
+++ b/ai-api-sites-table.xlsx
@@ -1287,7 +1287,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F38"/>
+  <dimension ref="A1:F39"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.81818181818182" defaultRowHeight="14"/>
   <cols>
     <col width="7" customWidth="1" style="9" min="1" max="1"/>
@@ -2259,30 +2259,60 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="n">
+      <c r="A38" s="0" t="n">
         <v>42</v>
       </c>
-      <c r="B38" t="inlineStr">
+      <c r="B38" s="0" t="inlineStr">
         <is>
           <t>modelport</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
+      <c r="C38" s="0" t="inlineStr">
         <is>
           <t>https://modelport.link/register?aff=KXEDZYFPJTH6</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr">
+      <c r="D38" s="0" t="inlineStr">
         <is>
           <t>GPT</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr">
+      <c r="E38" s="0" t="inlineStr">
         <is>
           <t>进群联系管理员可领取官倍 ¥3 站内体验额度，GPT 0.1x。</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr">
+      <c r="F38" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>43</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>JuCodex</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>https://jucodex.com/register?aff=6PXc</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>注册赠送;GPT;Codex</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>注册赠送3刀，GPT 0.05x。</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
         <is>
           <t>2026-07-30</t>
         </is>

</xml_diff>

<commit_message>
feat: add NexaRelay listing
</commit_message>
<xml_diff>
--- a/ai-api-sites-table.xlsx
+++ b/ai-api-sites-table.xlsx
@@ -1287,7 +1287,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F39"/>
+  <dimension ref="A1:F40"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.81818181818182" defaultRowHeight="14"/>
   <cols>
     <col width="7" customWidth="1" style="9" min="1" max="1"/>
@@ -2289,30 +2289,60 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="n">
+      <c r="A39" s="0" t="n">
         <v>43</v>
       </c>
-      <c r="B39" t="inlineStr">
+      <c r="B39" s="0" t="inlineStr">
         <is>
           <t>JuCodex</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
+      <c r="C39" s="0" t="inlineStr">
         <is>
           <t>https://jucodex.com/register?aff=6PXc</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr">
+      <c r="D39" s="0" t="inlineStr">
         <is>
           <t>注册赠送;GPT;Codex</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr">
+      <c r="E39" s="0" t="inlineStr">
         <is>
           <t>注册赠送3刀，GPT 0.05x。</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr">
+      <c r="F39" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>44</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>NexaRelay</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>https://api.nexarelay.com/register?aff=RVTTQ4NBGE6X</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>注册赠送</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>注册赠送3刀，0.2x 倍率，相当于15刀额度。</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
         <is>
           <t>2026-07-30</t>
         </is>

</xml_diff>

<commit_message>
feat: add 云核 listing
</commit_message>
<xml_diff>
--- a/ai-api-sites-table.xlsx
+++ b/ai-api-sites-table.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowWidth="24000" windowHeight="12080" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ai-api-sites-table" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="ai-api-sites-table" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -1287,7 +1287,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F40"/>
+  <dimension ref="A1:F41"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.81818181818182" defaultRowHeight="14"/>
   <cols>
     <col width="7" customWidth="1" style="9" min="1" max="1"/>
@@ -2319,32 +2319,58 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" t="n">
+      <c r="A40" s="0" t="n">
         <v>44</v>
       </c>
-      <c r="B40" t="inlineStr">
+      <c r="B40" s="0" t="inlineStr">
         <is>
           <t>NexaRelay</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
+      <c r="C40" s="0" t="inlineStr">
         <is>
           <t>https://api.nexarelay.com/register?aff=RVTTQ4NBGE6X</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr">
+      <c r="D40" s="0" t="inlineStr">
         <is>
           <t>注册赠送</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr">
+      <c r="E40" s="0" t="inlineStr">
         <is>
           <t>注册赠送3刀，0.2x 倍率，相当于15刀额度。</t>
         </is>
       </c>
-      <c r="F40" t="inlineStr">
+      <c r="F40" s="0" t="inlineStr">
         <is>
           <t>2026-07-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>45</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>云核</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>https://api.yunhe.one/sign-up?aff=fPZa</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr"/>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>注册送4刀，试营业plus 0.08倍率</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add Orbelis listing
</commit_message>
<xml_diff>
--- a/ai-api-sites-table.xlsx
+++ b/ai-api-sites-table.xlsx
@@ -1287,7 +1287,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F41"/>
+  <dimension ref="A1:F42"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.81818181818182" defaultRowHeight="14"/>
   <cols>
     <col width="7" customWidth="1" style="9" min="1" max="1"/>
@@ -2349,28 +2349,58 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" t="n">
+      <c r="A41" s="0" t="n">
         <v>45</v>
       </c>
-      <c r="B41" t="inlineStr">
+      <c r="B41" s="0" t="inlineStr">
         <is>
           <t>云核</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
+      <c r="C41" s="0" t="inlineStr">
         <is>
           <t>https://api.yunhe.one/sign-up?aff=fPZa</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr"/>
-      <c r="E41" t="inlineStr">
+      <c r="D41" s="0" t="inlineStr"/>
+      <c r="E41" s="0" t="inlineStr">
         <is>
           <t>注册送4刀，试营业plus 0.08倍率</t>
         </is>
       </c>
-      <c r="F41" t="inlineStr">
+      <c r="F41" s="0" t="inlineStr">
         <is>
           <t>2026-08-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>46</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Orbelis</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>https://nova.vcrauo.com/sign-up?aff=qhik</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>签到;注册赠送;DeepSeek;Gemini;GLM</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>支持 QQ 邮箱、GitHub 注册；Plus、Grok 特惠模型 0.04×，Plus 高速模型 0.08×；通过邀请码注册赠送 1 美元，进群或 Telegram 再领 1 美元，每日签到赠送 0.2 美元；DeepSeek 和 GLM 5.2 免费，另支持 Gemini。</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add 卡皮巴拉 API listing
</commit_message>
<xml_diff>
--- a/ai-api-sites-table.xlsx
+++ b/ai-api-sites-table.xlsx
@@ -1287,7 +1287,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F42"/>
+  <dimension ref="A1:F43"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.81818181818182" defaultRowHeight="14"/>
   <cols>
     <col width="7" customWidth="1" style="9" min="1" max="1"/>
@@ -2375,32 +2375,62 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" t="n">
+      <c r="A42" s="0" t="n">
         <v>46</v>
       </c>
-      <c r="B42" t="inlineStr">
+      <c r="B42" s="0" t="inlineStr">
         <is>
           <t>Orbelis</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
+      <c r="C42" s="0" t="inlineStr">
         <is>
           <t>https://nova.vcrauo.com/sign-up?aff=qhik</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr">
+      <c r="D42" s="0" t="inlineStr">
         <is>
           <t>签到;注册赠送;DeepSeek;Gemini;GLM</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr">
+      <c r="E42" s="0" t="inlineStr">
         <is>
           <t>支持 QQ 邮箱、GitHub 注册；Plus、Grok 特惠模型 0.04×，Plus 高速模型 0.08×；通过邀请码注册赠送 1 美元，进群或 Telegram 再领 1 美元，每日签到赠送 0.2 美元；DeepSeek 和 GLM 5.2 免费，另支持 Gemini。</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr">
+      <c r="F42" s="0" t="inlineStr">
         <is>
           <t>2026-08-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>47</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>卡皮巴拉 API</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>https://kapibala.asia/sign-up?aff=pEQ6</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>GPT</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>邀请码注册 22 刀，1 倍率</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add tabitoken listing
</commit_message>
<xml_diff>
--- a/ai-api-sites-table.xlsx
+++ b/ai-api-sites-table.xlsx
@@ -1287,7 +1287,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F43"/>
+  <dimension ref="A1:F44"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.81818181818182" defaultRowHeight="14"/>
   <cols>
     <col width="7" customWidth="1" style="9" min="1" max="1"/>
@@ -2405,32 +2405,62 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" t="n">
+      <c r="A43" s="0" t="n">
         <v>47</v>
       </c>
-      <c r="B43" t="inlineStr">
+      <c r="B43" s="0" t="inlineStr">
         <is>
           <t>卡皮巴拉 API</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
+      <c r="C43" s="0" t="inlineStr">
         <is>
           <t>https://kapibala.asia/sign-up?aff=pEQ6</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr">
+      <c r="D43" s="0" t="inlineStr">
         <is>
           <t>GPT</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr">
+      <c r="E43" s="0" t="inlineStr">
         <is>
           <t>邀请码注册 22 刀，1 倍率</t>
         </is>
       </c>
-      <c r="F43" t="inlineStr">
+      <c r="F43" s="0" t="inlineStr">
         <is>
           <t>2026-08-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>48</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>tabitoken</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>https://tabitoken.com/sign-up?aff=ySIl</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>注册赠送;邀请</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>实测注册赠送120刀，仅有CC模型，没有GPT；倍率1X；邀请1人奖励20刀。</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add straitapi listing
</commit_message>
<xml_diff>
--- a/ai-api-sites-table.xlsx
+++ b/ai-api-sites-table.xlsx
@@ -1287,7 +1287,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F44"/>
+  <dimension ref="A1:F45"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.81818181818182" defaultRowHeight="14"/>
   <cols>
     <col width="7" customWidth="1" style="9" min="1" max="1"/>
@@ -2435,32 +2435,62 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" t="n">
+      <c r="A44" s="0" t="n">
         <v>48</v>
       </c>
-      <c r="B44" t="inlineStr">
+      <c r="B44" s="0" t="inlineStr">
         <is>
           <t>tabitoken</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr">
+      <c r="C44" s="0" t="inlineStr">
         <is>
           <t>https://tabitoken.com/sign-up?aff=ySIl</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr">
+      <c r="D44" s="0" t="inlineStr">
         <is>
           <t>注册赠送;邀请</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr">
+      <c r="E44" s="0" t="inlineStr">
         <is>
           <t>实测注册赠送120刀，仅有CC模型，没有GPT；倍率1X；邀请1人奖励20刀。</t>
         </is>
       </c>
-      <c r="F44" t="inlineStr">
+      <c r="F44" s="0" t="inlineStr">
         <is>
           <t>2026-08-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>49</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>straitapi</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>https://straitapi.com/sign-up?aff=WU5M</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Claude;GPT</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>注册即到账 $2：通过邀请链接 + QQ邮箱注册，双方立刻各得 $2 额度！（⚠️必须使用QQ邮箱） 首充无门槛送 $3：充值 1 元也算首充！立得 $3 美金调用额度。 0.08X GPT 0.15X CLAUDE</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add ai.alsl.xyz listing
</commit_message>
<xml_diff>
--- a/ai-api-sites-table.xlsx
+++ b/ai-api-sites-table.xlsx
@@ -1287,7 +1287,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F45"/>
+  <dimension ref="A1:F46"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.81818181818182" defaultRowHeight="14"/>
   <cols>
     <col width="7" customWidth="1" style="9" min="1" max="1"/>
@@ -2465,32 +2465,62 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" t="n">
+      <c r="A45" s="0" t="n">
         <v>49</v>
       </c>
-      <c r="B45" t="inlineStr">
+      <c r="B45" s="0" t="inlineStr">
         <is>
           <t>straitapi</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr">
+      <c r="C45" s="0" t="inlineStr">
         <is>
           <t>https://straitapi.com/sign-up?aff=WU5M</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr">
+      <c r="D45" s="0" t="inlineStr">
         <is>
           <t>Claude;GPT</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr">
+      <c r="E45" s="0" t="inlineStr">
         <is>
           <t>注册即到账 $2：通过邀请链接 + QQ邮箱注册，双方立刻各得 $2 额度！（⚠️必须使用QQ邮箱） 首充无门槛送 $3：充值 1 元也算首充！立得 $3 美金调用额度。 0.08X GPT 0.15X CLAUDE</t>
         </is>
       </c>
-      <c r="F45" t="inlineStr">
+      <c r="F45" s="0" t="inlineStr">
         <is>
           <t>2026-08-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>50</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>ai.alsl.xyz</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>https://ai.alsl.xyz/register?aff=GP6NPUZHHEW8</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>GPT</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>注册送10刀新人体验gpt</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add sudoflow listing
</commit_message>
<xml_diff>
--- a/ai-api-sites-table.xlsx
+++ b/ai-api-sites-table.xlsx
@@ -1287,7 +1287,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F46"/>
+  <dimension ref="A1:F47"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.81818181818182" defaultRowHeight="14"/>
   <cols>
     <col width="7" customWidth="1" style="9" min="1" max="1"/>
@@ -2495,32 +2495,62 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="n">
+      <c r="A46" s="0" t="n">
         <v>50</v>
       </c>
-      <c r="B46" t="inlineStr">
+      <c r="B46" s="0" t="inlineStr">
         <is>
           <t>ai.alsl.xyz</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr">
+      <c r="C46" s="0" t="inlineStr">
         <is>
           <t>https://ai.alsl.xyz/register?aff=GP6NPUZHHEW8</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr">
+      <c r="D46" s="0" t="inlineStr">
         <is>
           <t>GPT</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr">
+      <c r="E46" s="0" t="inlineStr">
         <is>
           <t>注册送10刀新人体验gpt</t>
         </is>
       </c>
-      <c r="F46" t="inlineStr">
+      <c r="F46" s="0" t="inlineStr">
         <is>
           <t>2026-08-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>51</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>sudoflow</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>https://sudoflow.top/sign-up?aff=WLW8</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>GPT</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>AFF：https://sudoflow.top/sign-up?aff=WLW8 注册：QQ邮箱注册 倍率：0.065x的gpt 邀请：注册送7 刀</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
         </is>
       </c>
     </row>

</xml_diff>